<commit_message>
Revising the store emp upload template, additional assignment month column
</commit_message>
<xml_diff>
--- a/uploads/UPLOAD-TEMPLATE/STORE-EMP-UPLOAD-TEMPLATE.xlsx
+++ b/uploads/UPLOAD-TEMPLATE/STORE-EMP-UPLOAD-TEMPLATE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\akatok\Documents\INCENTIVES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\node proj\rest-api-nestjs\uploads\UPLOAD-TEMPLATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD402BE-B256-4D10-9AB4-5B6D9354678B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C7DDE92-7B20-4FB6-A1D6-3D8FBCEA582B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8DE630E0-0B89-4DDE-A92E-DF514EA9A919}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>STORE IFS</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>ACTIVE</t>
+  </si>
+  <si>
+    <t>ASSIGNMENT MONTH</t>
   </si>
 </sst>
 </file>
@@ -130,9 +133,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,25 +451,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAE589B1-C7BA-44D4-9E29-919A5892AA9B}">
-  <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,10 +511,13 @@
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>50000917</v>
       </c>
@@ -537,7 +545,10 @@
       <c r="K2" t="s">
         <v>17</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="2">
+        <v>46143</v>
+      </c>
+      <c r="O2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>